<commit_message>
The Apr27 package, its report and the SE parity fixture carry the stated boxes and the special rate pool
The Apr27 Self Employed package is regenerated from the changed templates
(Financialaccounts.xlsx and Fixedassets.xlsx; the other seven workbooks
came out byte-identical) and the advanced scenario reconciled against it:
RECONCILES, 899 of 905 checks passed, the six others the warnings that
carry a true figure (box 44's disposal loss, VitalTax's other-income
folds, box 73 leaving out box 71, and SA103S boxes 25 and 28 leaving out
the SE Full-only boxes). The derivation tests anchor their quarterly
depreciation on this report's P&L grid. The SE parity fixture is refreshed
for the new cells and checks; the other three products' fixtures moved
only in provenance, which the gate ignores, so they stay as they were.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Model: claude-opus-5[1m]
Claude-Session: https://claude.ai/code/session_01LfJ3xuWu14waiCm8mi7tEh
</commit_message>
<xml_diff>
--- a/packages/GB Accounts Self Employed 2027-04-05 (Apr27) Excel 2007/Financialaccounts.xlsx
+++ b/packages/GB Accounts Self Employed 2027-04-05 (Apr27) Excel 2007/Financialaccounts.xlsx
@@ -4521,6 +4521,9 @@
           <cell r="Z1">
             <v>0</v>
           </cell>
+          <cell r="AC1">
+            <v>0</v>
+          </cell>
         </row>
         <row r="38">
           <cell r="R38" t="str">
@@ -8266,10 +8269,16 @@
         <v>46173</v>
       </c>
       <c r="C6" s="147"/>
-      <c r="D6" s="147"/>
+      <c r="D6" s="450" t="inlineStr">
+        <is>
+          <t>Special rate writing down allowance</t>
+        </is>
+      </c>
       <c r="E6" s="147"/>
       <c r="F6" s="147"/>
-      <c r="G6" s="146"/>
+      <c r="G6" s="148">
+        <v>0.06</v>
+      </c>
       <c r="H6" s="147"/>
       <c r="I6" s="450" t="s">
         <v>141</v>
@@ -11272,7 +11281,7 @@
         <v>51</v>
       </c>
       <c r="O80" s="356">
-        <f>IF(([1]Schedule!$R$1+[1]Schedule!$Y$1)&gt;0,[1]Schedule!$R$1+[1]Schedule!$Y$1,0)</f>
+        <f>IF(([1]Schedule!$R$1+[1]Schedule!$Y$1+[1]Schedule!$AC$1)&gt;0,[1]Schedule!$R$1+[1]Schedule!$Y$1+[1]Schedule!$AC$1,0)</f>
         <v>0</v>
       </c>
       <c r="P80" s="357"/>
@@ -17234,7 +17243,10 @@
       <c r="C147" s="217" t="s">
         <v>51</v>
       </c>
-      <c r="D147" s="356"/>
+      <c r="D147" s="356">
+        <f>[1]Schedule!$AC$1</f>
+        <v>0</v>
+      </c>
       <c r="E147" s="357"/>
       <c r="F147" s="358"/>
       <c r="G147" s="218" t="s">
@@ -30585,7 +30597,7 @@
         <v>86</v>
       </c>
       <c r="C38" s="128">
-        <f>[1]Schedule!$Q$1+[1]Schedule!$R$1+[1]Schedule!$Y$1-[1]Schedule!$Z$1</f>
+        <f>[1]Schedule!$Q$1+[1]Schedule!$R$1+[1]Schedule!$AC$1+[1]Schedule!$Y$1-[1]Schedule!$Z$1</f>
         <v>0</v>
       </c>
       <c r="D38" s="23"/>

</xml_diff>